<commit_message>
matching up population names
</commit_message>
<xml_diff>
--- a/Data/location<->population_key.xlsx
+++ b/Data/location<->population_key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dshizuka2/Documents/GitHub/BARS_phenotypic_integration/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453E3664-76F8-3149-A34D-4F00DF0FDE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42998C9C-83E8-BB4E-B9E6-30A715574B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="44800" windowHeight="23040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="24080" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="location&lt;-&gt;population_key" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10914" uniqueCount="1776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10985" uniqueCount="1779">
   <si>
     <t>location</t>
   </si>
@@ -5617,6 +5617,15 @@
   </si>
   <si>
     <t>Boulder</t>
+  </si>
+  <si>
+    <t>other_pop_name</t>
+  </si>
+  <si>
+    <t>khingui</t>
+  </si>
+  <si>
+    <t>takecha</t>
   </si>
 </sst>
 </file>
@@ -6045,7 +6054,9 @@
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1"/>
+      <c r="G1" s="1" t="s">
+        <v>1776</v>
+      </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -6087,6 +6098,9 @@
       <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G2" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" spans="1:28" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -6107,6 +6121,9 @@
       <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4" spans="1:28" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -6127,6 +6144,9 @@
       <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G4" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:28" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -6147,6 +6167,9 @@
       <c r="F5" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G5" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:28" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
@@ -6167,6 +6190,9 @@
       <c r="F6" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G6" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="1:28" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
@@ -6187,6 +6213,9 @@
       <c r="F7" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="G7" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:28" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -6207,6 +6236,9 @@
       <c r="F8" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="G8" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9" spans="1:28" ht="15.75" customHeight="1">
       <c r="A9" s="2" t="s">
@@ -6227,6 +6259,9 @@
       <c r="F9" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="G9" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="10" spans="1:28" ht="15.75" customHeight="1">
       <c r="A10" s="2" t="s">
@@ -6247,6 +6282,9 @@
       <c r="F10" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="G10" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="11" spans="1:28" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -6267,6 +6305,9 @@
       <c r="F11" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="G11" s="2" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="12" spans="1:28" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="s">
@@ -6287,6 +6328,9 @@
       <c r="F12" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="G12" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="13" spans="1:28" ht="15.75" customHeight="1">
       <c r="A13" s="2" t="s">
@@ -6307,6 +6351,9 @@
       <c r="F13" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="G13" s="2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="14" spans="1:28" ht="15.75" customHeight="1">
       <c r="A14" s="2" t="s">
@@ -6327,6 +6374,9 @@
       <c r="F14" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="G14" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="15" spans="1:28" ht="15.75" customHeight="1">
       <c r="A15" s="2" t="s">
@@ -6347,6 +6397,9 @@
       <c r="F15" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="G15" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="16" spans="1:28" ht="15.75" customHeight="1">
       <c r="A16" s="2" t="s">
@@ -6367,8 +6420,11 @@
       <c r="F16" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G16" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>40</v>
       </c>
@@ -6387,8 +6443,11 @@
       <c r="F17" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G17" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -6407,8 +6466,11 @@
       <c r="F18" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G18" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>44</v>
       </c>
@@ -6427,8 +6489,11 @@
       <c r="F19" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G19" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>47</v>
       </c>
@@ -6447,8 +6512,11 @@
       <c r="F20" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G20" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
@@ -6467,8 +6535,11 @@
       <c r="F21" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G21" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>51</v>
       </c>
@@ -6487,8 +6558,11 @@
       <c r="F22" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G22" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>53</v>
       </c>
@@ -6507,8 +6581,11 @@
       <c r="F23" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G23" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>55</v>
       </c>
@@ -6527,8 +6604,11 @@
       <c r="F24" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G24" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>57</v>
       </c>
@@ -6547,8 +6627,11 @@
       <c r="F25" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G25" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>60</v>
       </c>
@@ -6567,8 +6650,11 @@
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G26" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>62</v>
       </c>
@@ -6587,8 +6673,11 @@
       <c r="F27" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G27" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>65</v>
       </c>
@@ -6607,8 +6696,11 @@
       <c r="F28" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G28" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>68</v>
       </c>
@@ -6627,8 +6719,11 @@
       <c r="F29" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G29" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>70</v>
       </c>
@@ -6647,8 +6742,11 @@
       <c r="F30" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G30" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>72</v>
       </c>
@@ -6667,8 +6765,11 @@
       <c r="F31" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G31" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>74</v>
       </c>
@@ -6687,8 +6788,11 @@
       <c r="F32" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G32" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>76</v>
       </c>
@@ -6707,8 +6811,11 @@
       <c r="F33" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G33" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>78</v>
       </c>
@@ -6727,8 +6834,11 @@
       <c r="F34" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G34" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>80</v>
       </c>
@@ -6747,8 +6857,11 @@
       <c r="F35" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G35" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>82</v>
       </c>
@@ -6767,8 +6880,11 @@
       <c r="F36" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G36" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>84</v>
       </c>
@@ -6787,8 +6903,11 @@
       <c r="F37" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G37" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>86</v>
       </c>
@@ -6807,8 +6926,11 @@
       <c r="F38" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G38" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>88</v>
       </c>
@@ -6827,8 +6949,11 @@
       <c r="F39" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G39" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>90</v>
       </c>
@@ -6847,8 +6972,11 @@
       <c r="F40" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G40" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>92</v>
       </c>
@@ -6867,8 +6995,11 @@
       <c r="F41" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G41" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>94</v>
       </c>
@@ -6887,8 +7018,11 @@
       <c r="F42" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G42" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>96</v>
       </c>
@@ -6907,8 +7041,11 @@
       <c r="F43" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G43" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>98</v>
       </c>
@@ -6927,8 +7064,11 @@
       <c r="F44" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G44" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>100</v>
       </c>
@@ -6947,8 +7087,11 @@
       <c r="F45" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G45" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>103</v>
       </c>
@@ -6967,8 +7110,11 @@
       <c r="F46" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G46" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>105</v>
       </c>
@@ -6987,8 +7133,11 @@
       <c r="F47" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G47" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>107</v>
       </c>
@@ -7007,8 +7156,11 @@
       <c r="F48" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G48" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="15.75" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>109</v>
       </c>
@@ -7027,8 +7179,11 @@
       <c r="F49" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G49" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15.75" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>111</v>
       </c>
@@ -7047,8 +7202,11 @@
       <c r="F50" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G50" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>113</v>
       </c>
@@ -7067,8 +7225,11 @@
       <c r="F51" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G51" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="15.75" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>115</v>
       </c>
@@ -7087,8 +7248,11 @@
       <c r="F52" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G52" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="15.75" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>117</v>
       </c>
@@ -7107,8 +7271,11 @@
       <c r="F53" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G53" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15.75" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>119</v>
       </c>
@@ -7127,8 +7294,11 @@
       <c r="F54" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G54" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="15.75" customHeight="1">
       <c r="A55" s="2" t="s">
         <v>121</v>
       </c>
@@ -7147,8 +7317,11 @@
       <c r="F55" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G55" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="15.75" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>123</v>
       </c>
@@ -7167,8 +7340,11 @@
       <c r="F56" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G56" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="15.75" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>125</v>
       </c>
@@ -7187,8 +7363,11 @@
       <c r="F57" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G57" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="15.75" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>127</v>
       </c>
@@ -7207,8 +7386,11 @@
       <c r="F58" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G58" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="15.75" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>129</v>
       </c>
@@ -7227,8 +7409,11 @@
       <c r="F59" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G59" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="15.75" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>131</v>
       </c>
@@ -7247,8 +7432,11 @@
       <c r="F60" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G60" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="15.75" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>133</v>
       </c>
@@ -7267,8 +7455,11 @@
       <c r="F61" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G61" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="15.75" customHeight="1">
       <c r="A62" s="2" t="s">
         <v>135</v>
       </c>
@@ -7287,8 +7478,11 @@
       <c r="F62" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G62" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="15.75" customHeight="1">
       <c r="A63" s="2" t="s">
         <v>137</v>
       </c>
@@ -7307,8 +7501,11 @@
       <c r="F63" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G63" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="15.75" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>139</v>
       </c>
@@ -7327,8 +7524,11 @@
       <c r="F64" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G64" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="15.75" customHeight="1">
       <c r="A65" s="2" t="s">
         <v>141</v>
       </c>
@@ -7347,8 +7547,11 @@
       <c r="F65" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G65" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="15.75" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>143</v>
       </c>
@@ -7367,8 +7570,11 @@
       <c r="F66" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G66" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="15.75" customHeight="1">
       <c r="A67" s="2" t="s">
         <v>145</v>
       </c>
@@ -7387,8 +7593,11 @@
       <c r="F67" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G67" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="15.75" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>147</v>
       </c>
@@ -7407,8 +7616,11 @@
       <c r="F68" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G68" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="15.75" customHeight="1">
       <c r="A69" s="2" t="s">
         <v>149</v>
       </c>
@@ -7427,8 +7639,11 @@
       <c r="F69" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" ht="15.75" customHeight="1">
+      <c r="G69" s="2" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="15.75" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>151</v>
       </c>
@@ -7447,8 +7662,11 @@
       <c r="F70" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" ht="13">
+      <c r="G70" s="2" t="s">
+        <v>1777</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="13">
       <c r="A71" s="2" t="s">
         <v>153</v>
       </c>
@@ -7466,6 +7684,9 @@
       </c>
       <c r="F71" s="2" t="s">
         <v>67</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>1778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>